<commit_message>
Prepare declarations directly from folder workbooks with saved applicant contact
</commit_message>
<xml_diff>
--- a/docs/intake-template.xlsx
+++ b/docs/intake-template.xlsx
@@ -842,17 +842,29 @@
       <c r="C43" s="2" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n"/>
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>실적접수번호</t>
+        </is>
+      </c>
       <c r="B44" s="2" t="n"/>
       <c r="C44" s="2" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n"/>
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>실적신청번호</t>
+        </is>
+      </c>
       <c r="B45" s="2" t="n"/>
       <c r="C45" s="2" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n"/>
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>실적신청일</t>
+        </is>
+      </c>
       <c r="B46" s="2" t="n"/>
       <c r="C46" s="2" t="n"/>
     </row>

</xml_diff>

<commit_message>
Read declaration workbooks directly from shipment folders (1.3.0)
* Prepare declarations directly from folder workbooks with saved applicant contact

* Show the installed version consistently on the home screen
</commit_message>
<xml_diff>
--- a/docs/intake-template.xlsx
+++ b/docs/intake-template.xlsx
@@ -842,17 +842,29 @@
       <c r="C43" s="2" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n"/>
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>실적접수번호</t>
+        </is>
+      </c>
       <c r="B44" s="2" t="n"/>
       <c r="C44" s="2" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n"/>
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>실적신청번호</t>
+        </is>
+      </c>
       <c r="B45" s="2" t="n"/>
       <c r="C45" s="2" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n"/>
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>실적신청일</t>
+        </is>
+      </c>
       <c r="B46" s="2" t="n"/>
       <c r="C46" s="2" t="n"/>
     </row>

</xml_diff>